<commit_message>
Align DSA2026 assignment 2 model answer with revised problem text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dsa/DSA2026_kadai2_模範解答.xlsx
+++ b/dsa/DSA2026_kadai2_模範解答.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -458,281 +458,41 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>三条市</t>
+          <t>上越市</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>88396</v>
+        <v>176481</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>柏崎市</t>
+          <t>新発田市</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74728</v>
+        <v>89570</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>新発田市</t>
+          <t>三条市</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>89570</v>
+        <v>88396</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>小千谷市</t>
+          <t>その他</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31408</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>加茂市</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>23024</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>十日町市</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>44509</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>見附市</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>36613</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>村上市</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>51422</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>燕市</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>73706</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>糸魚川市</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>36519</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>妙高市</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>27860</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>五泉市</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>43481</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>上越市</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>176481</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>阿賀野市</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>37503</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>佐渡市</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>45378</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>魚沼市</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>31026</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>南魚沼市</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>51184</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>胎内市</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>26235</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>聖籠町</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>14071</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>弥彦村</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>7114</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>田上町</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>10287</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>阿賀町</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>8338</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>出雲崎町</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3597</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>湯沢町</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>7510</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>津南町</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>7959</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>刈羽村</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>4318</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>関川村</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>4396</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>粟島浦村</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>303</v>
+        <v>702489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>